<commit_message>
Added gradient boosting tutorial
</commit_message>
<xml_diff>
--- a/4. Supervised Learning (modeling and evaluation)/MLPClassifier Excel inference.xlsx
+++ b/4. Supervised Learning (modeling and evaluation)/MLPClassifier Excel inference.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eugenio/Documents/Notebooks_ArtificialIntelligence/4. Supervised Learning (modeling and evaluation)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4345FFF8-C805-F04B-93B9-FD5A738EE75D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7A7B577-5A62-B341-8F44-9CFF3BD07536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17780" xr2:uid="{41000640-C45C-B943-AC1A-91C2BB07B558}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -228,7 +228,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -236,10 +236,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -248,12 +251,10 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -663,14 +664,14 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="2" spans="1:100" x14ac:dyDescent="0.2">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
     </row>
     <row r="3" spans="1:100" x14ac:dyDescent="0.2">
       <c r="A3">
@@ -693,12 +694,12 @@
       </c>
     </row>
     <row r="5" spans="1:100" x14ac:dyDescent="0.2">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
     </row>
     <row r="6" spans="1:100" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
@@ -2815,12 +2816,12 @@
       </c>
     </row>
     <row r="14" spans="1:100" x14ac:dyDescent="0.2">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
     </row>
     <row r="15" spans="1:100" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
@@ -2831,12 +2832,12 @@
       <c r="A16">
         <v>0.2111082486469878</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
     </row>
     <row r="17" spans="1:102" x14ac:dyDescent="0.2">
       <c r="A17">
@@ -3153,15 +3154,15 @@
       <c r="A19">
         <v>-0.18211426198386671</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
     </row>
     <row r="20" spans="1:102" x14ac:dyDescent="0.2">
       <c r="A20">
@@ -3478,11 +3479,11 @@
       <c r="A22">
         <v>-7.3572614846321603E-3</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
     </row>
     <row r="23" spans="1:102" x14ac:dyDescent="0.2">
       <c r="A23">
@@ -3898,12 +3899,12 @@
       <c r="A25">
         <v>0.20117547107948411</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
     </row>
     <row r="26" spans="1:102" x14ac:dyDescent="0.2">
       <c r="A26">
@@ -34678,15 +34679,15 @@
       </c>
     </row>
     <row r="128" spans="1:102" x14ac:dyDescent="0.2">
-      <c r="C128" s="7" t="s">
+      <c r="C128" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D128" s="7"/>
-      <c r="E128" s="7"/>
-      <c r="F128" s="7"/>
-      <c r="G128" s="7"/>
-      <c r="H128" s="7"/>
-      <c r="I128" s="7"/>
+      <c r="D128" s="8"/>
+      <c r="E128" s="8"/>
+      <c r="F128" s="8"/>
+      <c r="G128" s="8"/>
+      <c r="H128" s="8"/>
+      <c r="I128" s="8"/>
     </row>
     <row r="129" spans="1:104" x14ac:dyDescent="0.2">
       <c r="C129" cm="1">
@@ -34992,26 +34993,26 @@
       </c>
     </row>
     <row r="131" spans="1:104" x14ac:dyDescent="0.2">
-      <c r="A131" s="9" t="s">
+      <c r="A131" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B131" s="9"/>
-      <c r="C131" s="9"/>
+      <c r="B131" s="6"/>
+      <c r="C131" s="6"/>
     </row>
     <row r="132" spans="1:104" x14ac:dyDescent="0.2">
       <c r="C132" s="1">
         <v>0</v>
       </c>
-      <c r="E132" s="8" t="s">
+      <c r="E132" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F132" s="8"/>
-      <c r="G132" s="8"/>
-      <c r="H132" s="8"/>
-      <c r="I132" s="8"/>
-      <c r="J132" s="8"/>
-      <c r="K132" s="8"/>
-      <c r="L132" s="8"/>
+      <c r="F132" s="9"/>
+      <c r="G132" s="9"/>
+      <c r="H132" s="9"/>
+      <c r="I132" s="9"/>
+      <c r="J132" s="9"/>
+      <c r="K132" s="9"/>
+      <c r="L132" s="9"/>
     </row>
     <row r="133" spans="1:104" x14ac:dyDescent="0.2">
       <c r="C133">
@@ -35328,11 +35329,11 @@
       <c r="C135">
         <v>-0.13894647915350899</v>
       </c>
-      <c r="E135" s="5" t="s">
+      <c r="E135" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="F135" s="5"/>
-      <c r="G135" s="5"/>
+      <c r="F135" s="10"/>
+      <c r="G135" s="10"/>
     </row>
     <row r="136" spans="1:104" x14ac:dyDescent="0.2">
       <c r="C136">
@@ -35748,12 +35749,12 @@
       <c r="C138">
         <v>-4.5757920258084946E-3</v>
       </c>
-      <c r="E138" s="6" t="s">
+      <c r="E138" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F138" s="6"/>
-      <c r="G138" s="6"/>
-      <c r="H138" s="6"/>
+      <c r="F138" s="5"/>
+      <c r="G138" s="5"/>
+      <c r="H138" s="5"/>
     </row>
     <row r="139" spans="1:104" x14ac:dyDescent="0.2">
       <c r="C139">
@@ -35782,15 +35783,15 @@
       <c r="G140">
         <v>-7.127601824142453E-2</v>
       </c>
-      <c r="I140" s="7" t="s">
+      <c r="I140" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="J140" s="7"/>
-      <c r="K140" s="7"/>
-      <c r="L140" s="7"/>
-      <c r="M140" s="7"/>
-      <c r="N140" s="7"/>
-      <c r="O140" s="7"/>
+      <c r="J140" s="8"/>
+      <c r="K140" s="8"/>
+      <c r="L140" s="8"/>
+      <c r="M140" s="8"/>
+      <c r="N140" s="8"/>
+      <c r="O140" s="8"/>
     </row>
     <row r="141" spans="1:104" x14ac:dyDescent="0.2">
       <c r="C141">
@@ -35843,11 +35844,11 @@
       <c r="G143">
         <v>-2.5623923656746058E-6</v>
       </c>
-      <c r="I143" s="9" t="s">
+      <c r="I143" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="J143" s="9"/>
-      <c r="K143" s="9"/>
+      <c r="J143" s="6"/>
+      <c r="K143" s="6"/>
     </row>
     <row r="144" spans="1:104" x14ac:dyDescent="0.2">
       <c r="C144">
@@ -35944,16 +35945,16 @@
       <c r="G149">
         <v>-0.20016515315201391</v>
       </c>
-      <c r="I149" s="8" t="s">
+      <c r="I149" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="J149" s="8"/>
-      <c r="K149" s="8"/>
-      <c r="L149" s="8"/>
-      <c r="M149" s="8"/>
-      <c r="N149" s="8"/>
-      <c r="O149" s="8"/>
-      <c r="P149" s="8"/>
+      <c r="J149" s="9"/>
+      <c r="K149" s="9"/>
+      <c r="L149" s="9"/>
+      <c r="M149" s="9"/>
+      <c r="N149" s="9"/>
+      <c r="O149" s="9"/>
+      <c r="P149" s="9"/>
       <c r="R149" s="2"/>
     </row>
     <row r="150" spans="3:18" x14ac:dyDescent="0.2">
@@ -36007,11 +36008,11 @@
       <c r="G152">
         <v>0.1192830653186049</v>
       </c>
-      <c r="I152" s="5" t="s">
+      <c r="I152" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="J152" s="5"/>
-      <c r="K152" s="5"/>
+      <c r="J152" s="10"/>
+      <c r="K152" s="10"/>
     </row>
     <row r="153" spans="3:18" x14ac:dyDescent="0.2">
       <c r="C153">
@@ -36026,7 +36027,7 @@
       <c r="G153">
         <v>3.122834673913675E-3</v>
       </c>
-      <c r="I153">
+      <c r="I153" s="11">
         <f>EXP(I150)/(EXP(I150)+EXP(J150)+EXP(K150))</f>
         <v>0.99999815544471715</v>
       </c>
@@ -37233,11 +37234,6 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A14:D14"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="C16:F16"/>
-    <mergeCell ref="C19:I19"/>
     <mergeCell ref="I152:K152"/>
     <mergeCell ref="C22:E22"/>
     <mergeCell ref="C25:F25"/>
@@ -37249,6 +37245,11 @@
     <mergeCell ref="I140:O140"/>
     <mergeCell ref="I149:P149"/>
     <mergeCell ref="I143:K143"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="C16:F16"/>
+    <mergeCell ref="C19:I19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Add Streamlit app UIDE
</commit_message>
<xml_diff>
--- a/4. Supervised Learning (modeling and evaluation)/MLPClassifier Excel inference.xlsx
+++ b/4. Supervised Learning (modeling and evaluation)/MLPClassifier Excel inference.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eugenio/Documents/Notebooks_ArtificialIntelligence/4. Supervised Learning (modeling and evaluation)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7A7B577-5A62-B341-8F44-9CFF3BD07536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDFEBFA3-7BBD-FC4F-9751-5B85320F9ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17780" xr2:uid="{41000640-C45C-B943-AC1A-91C2BB07B558}"/>
   </bookViews>
@@ -236,7 +236,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -245,16 +255,6 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -664,14 +664,14 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="2" spans="1:100" x14ac:dyDescent="0.2">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
     </row>
     <row r="3" spans="1:100" x14ac:dyDescent="0.2">
       <c r="A3">
@@ -694,12 +694,12 @@
       </c>
     </row>
     <row r="5" spans="1:100" x14ac:dyDescent="0.2">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
     </row>
     <row r="6" spans="1:100" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
@@ -2816,12 +2816,12 @@
       </c>
     </row>
     <row r="14" spans="1:100" x14ac:dyDescent="0.2">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
     </row>
     <row r="15" spans="1:100" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
@@ -3479,11 +3479,11 @@
       <c r="A22">
         <v>-7.3572614846321603E-3</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
     </row>
     <row r="23" spans="1:102" x14ac:dyDescent="0.2">
       <c r="A23">
@@ -3899,12 +3899,12 @@
       <c r="A25">
         <v>0.20117547107948411</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
     </row>
     <row r="26" spans="1:102" x14ac:dyDescent="0.2">
       <c r="A26">
@@ -34993,11 +34993,11 @@
       </c>
     </row>
     <row r="131" spans="1:104" x14ac:dyDescent="0.2">
-      <c r="A131" s="6" t="s">
+      <c r="A131" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B131" s="6"/>
-      <c r="C131" s="6"/>
+      <c r="B131" s="10"/>
+      <c r="C131" s="10"/>
     </row>
     <row r="132" spans="1:104" x14ac:dyDescent="0.2">
       <c r="C132" s="1">
@@ -35329,11 +35329,11 @@
       <c r="C135">
         <v>-0.13894647915350899</v>
       </c>
-      <c r="E135" s="10" t="s">
+      <c r="E135" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F135" s="10"/>
-      <c r="G135" s="10"/>
+      <c r="F135" s="6"/>
+      <c r="G135" s="6"/>
     </row>
     <row r="136" spans="1:104" x14ac:dyDescent="0.2">
       <c r="C136">
@@ -35749,12 +35749,12 @@
       <c r="C138">
         <v>-4.5757920258084946E-3</v>
       </c>
-      <c r="E138" s="5" t="s">
+      <c r="E138" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="F138" s="5"/>
-      <c r="G138" s="5"/>
-      <c r="H138" s="5"/>
+      <c r="F138" s="7"/>
+      <c r="G138" s="7"/>
+      <c r="H138" s="7"/>
     </row>
     <row r="139" spans="1:104" x14ac:dyDescent="0.2">
       <c r="C139">
@@ -35844,11 +35844,11 @@
       <c r="G143">
         <v>-2.5623923656746058E-6</v>
       </c>
-      <c r="I143" s="6" t="s">
+      <c r="I143" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="J143" s="6"/>
-      <c r="K143" s="6"/>
+      <c r="J143" s="10"/>
+      <c r="K143" s="10"/>
     </row>
     <row r="144" spans="1:104" x14ac:dyDescent="0.2">
       <c r="C144">
@@ -36008,11 +36008,11 @@
       <c r="G152">
         <v>0.1192830653186049</v>
       </c>
-      <c r="I152" s="10" t="s">
+      <c r="I152" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="J152" s="10"/>
-      <c r="K152" s="10"/>
+      <c r="J152" s="6"/>
+      <c r="K152" s="6"/>
     </row>
     <row r="153" spans="3:18" x14ac:dyDescent="0.2">
       <c r="C153">
@@ -36027,7 +36027,7 @@
       <c r="G153">
         <v>3.122834673913675E-3</v>
       </c>
-      <c r="I153" s="11">
+      <c r="I153" s="5">
         <f>EXP(I150)/(EXP(I150)+EXP(J150)+EXP(K150))</f>
         <v>0.99999815544471715</v>
       </c>
@@ -37234,6 +37234,11 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="C16:F16"/>
+    <mergeCell ref="C19:I19"/>
     <mergeCell ref="I152:K152"/>
     <mergeCell ref="C22:E22"/>
     <mergeCell ref="C25:F25"/>
@@ -37245,11 +37250,6 @@
     <mergeCell ref="I140:O140"/>
     <mergeCell ref="I149:P149"/>
     <mergeCell ref="I143:K143"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A14:D14"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="C16:F16"/>
-    <mergeCell ref="C19:I19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>